<commit_message>
feat(data): add test spreadsheets with Caio's contact details for campaign testing
</commit_message>
<xml_diff>
--- a/planilha_teste.xlsx
+++ b/planilha_teste.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Leads" sheetId="1" r:id="rId1"/>
+    <sheet name="Leads_Vero" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,35 +397,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>nome</v>
+        <v>NOME</v>
       </c>
       <c r="B1" t="str">
-        <v>cpf</v>
+        <v>TELEFONE</v>
       </c>
       <c r="C1" t="str">
-        <v>telefone</v>
+        <v>CPF</v>
       </c>
       <c r="D1" t="str">
-        <v>valor</v>
+        <v>EMAIL</v>
       </c>
       <c r="E1" t="str">
-        <v>vencimento</v>
+        <v>VAL_NOMINAL</v>
       </c>
       <c r="F1" t="str">
-        <v>linha_digitavel</v>
+        <v>VENCIMENTO</v>
       </c>
       <c r="G1" t="str">
-        <v>dias_atraso</v>
+        <v>LINHA_DIGITAVEL</v>
       </c>
       <c r="H1" t="str">
-        <v>status_internet</v>
+        <v>DIAS_ATRASO</v>
       </c>
       <c r="I1" t="str">
-        <v>email</v>
+        <v>STATUS_INTERNET</v>
       </c>
     </row>
     <row r="2">
@@ -433,33 +433,62 @@
         <v>Caio Vicente</v>
       </c>
       <c r="B2" t="str">
+        <v>21984354821</v>
+      </c>
+      <c r="C2" t="str">
         <v>123.456.789-00</v>
       </c>
-      <c r="C2" t="str">
-        <v>5521981811077</v>
-      </c>
       <c r="D2" t="str">
-        <v>189,90</v>
-      </c>
-      <c r="E2" t="str">
+        <v>caiovicenteti@gmail.com</v>
+      </c>
+      <c r="E2">
+        <v>149.9</v>
+      </c>
+      <c r="F2" t="str">
         <v>10/09/2026</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
+        <v>34191000070000000000400000000000190000000014990</v>
+      </c>
+      <c r="H2">
+        <v>4</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Ativo</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Caio Renato</v>
+      </c>
+      <c r="B3" t="str">
+        <v>21981811077</v>
+      </c>
+      <c r="C3" t="str">
+        <v>987.654.321-99</v>
+      </c>
+      <c r="D3" t="str">
+        <v>caiovicenteti@gmail.com</v>
+      </c>
+      <c r="E3">
+        <v>189.9</v>
+      </c>
+      <c r="F3" t="str">
+        <v>05/09/2026</v>
+      </c>
+      <c r="G3" t="str">
         <v>84670000001743590024020902405020130000000000</v>
       </c>
-      <c r="G2" t="str">
-        <v>12</v>
-      </c>
-      <c r="H2" t="str">
-        <v>BLOQUEADO</v>
-      </c>
-      <c r="I2" t="str">
-        <v>caio.vicente@vero.com.br</v>
+      <c r="H3">
+        <v>9</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Bloqueio Parcial</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>